<commit_message>
dados: D001 como identificador e prefixo do nome do conjunto
</commit_message>
<xml_diff>
--- a/data-raw/isoproteica_bagre/bagres_para_revisao.xlsx
+++ b/data-raw/isoproteica_bagre/bagres_para_revisao.xlsx
@@ -270,10 +270,10 @@
     <t>ANOVA 1 fator; Welch; Kruskal-Wallis. Adequação depende da revisão do desenho e dos pressupostos.</t>
   </si>
   <si>
-    <t>Identificador D-xxx</t>
-  </si>
-  <si>
-    <t>D-001 — bagre_racao_isoproteica</t>
+    <t>Identificador Dxxx</t>
+  </si>
+  <si>
+    <t>D001 — D001_bagre_racao_isoproteica</t>
   </si>
   <si>
     <t>Data da cópia</t>

</xml_diff>